<commit_message>
Standardize QC reports and complete release evidence
</commit_message>
<xml_diff>
--- a/examples/qualibact_ecoli/fail_only/report/report.xlsx
+++ b/examples/qualibact_ecoli/fail_only/report/report.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,67 +436,87 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>all_checks_passed</t>
+          <t>speccheck_qc</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>qualibact_compat_tier</t>
+          <t>qualibact_qc</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>historical_qualibact_qc</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>reason_summary</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>species</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>species_confidence</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>n50</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>contigs</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>genome_size</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>gc_percent</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>completeness</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>contamination</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>top_species</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>top_abundance</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>reason_summary</t>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>top_abundance_percent</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>threshold_source</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>report_schema_version</t>
         </is>
       </c>
     </row>
@@ -513,7 +533,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -521,45 +541,53 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>19474</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>522</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>4153626</v>
       </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
         <v>50.8872</v>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>100</v>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>0.25</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="N2" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
+      <c r="Q2" t="n">
+        <v>75</v>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -576,7 +604,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -584,45 +612,53 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>126621</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
         <v>679</v>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>5738641</v>
       </c>
-      <c r="J3" t="n">
+      <c r="L3" t="n">
         <v>50.5585</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>100</v>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>0.4</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="N3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
+      <c r="Q3" t="n">
+        <v>75</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -637,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -653,67 +689,87 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>all_checks_passed</t>
+          <t>speccheck_qc</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>qualibact_compat_tier</t>
+          <t>qualibact_qc</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>historical_qualibact_qc</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>reason_summary</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>species</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>species_confidence</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>n50</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>contigs</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>genome_size</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>gc_percent</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>completeness</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>contamination</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>top_species</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>top_abundance</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>reason_summary</t>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>top_abundance_percent</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>threshold_source</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>report_schema_version</t>
         </is>
       </c>
     </row>
@@ -730,7 +786,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -738,45 +794,53 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>19474</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>522</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>4153626</v>
       </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
         <v>50.8872</v>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>100</v>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>0.25</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="N2" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
+      <c r="Q2" t="n">
+        <v>75</v>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -793,7 +857,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -801,45 +865,53 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>126621</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
         <v>679</v>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>5738641</v>
       </c>
-      <c r="J3" t="n">
+      <c r="L3" t="n">
         <v>50.5585</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>100</v>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>0.4</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="N3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
+      <c r="Q3" t="n">
+        <v>75</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -854,7 +926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO3"/>
+  <dimension ref="A1:AX3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -865,202 +937,247 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Checkm.Completeness.check</t>
+          <t>overall_qc</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Checkm.Contamination.check</t>
+          <t>speccheck_qc</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Quast.# contigs (&gt;= 0 bp).check</t>
+          <t>qualibact_qc</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Quast.GC (%).check</t>
+          <t>historical_qualibact_qc</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Quast.N50.check</t>
+          <t>reason_summary</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Quast.Total length (&gt;= 0 bp).check</t>
+          <t>species</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Checkm.# contigs</t>
+          <t>species_confidence</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>n50</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>contigs</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>genome_size</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>gc_percent</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>completeness</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>contamination</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>top_species</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>top_abundance_percent</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>threshold_source</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>report_schema_version</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Speciator.qc_status</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Speciator.confidence</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Speciator.speciesName</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Sylph.qc_status</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Sylph.number_of_genomes</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Sylph.top_abundance_percent</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Sylph.top_species</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Quast.qc_status</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Quast.# contigs (&gt;= 0 bp)</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Quast.# contigs (&gt;= 0 bp).status</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>Quast.GC (%)</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>Quast.GC (%).status</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Quast.Largest contig</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Quast.N50</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>Quast.N50.status</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>Quast.Total length (&gt;= 0 bp)</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>Quast.Total length (&gt;= 0 bp).status</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>Checkm.qc_status</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
           <t>Checkm.Completeness</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>Checkm.Completeness.status</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Checkm.Contamination</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Checkm.GC</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Checkm.Genome size (bp)</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Checkm.N50 (scaffolds)</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>Checkm.Contamination.status</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>Checkm.Contig_N50</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>Checkm.GC_Content</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>Checkm.Genome_Size</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
         <is>
           <t>Checkm.Total_Coding_Sequences</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Checkm.all_checks_passed</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Quast.# contigs (&gt;= 0 bp)</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Quast.GC (%)</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Quast.Largest contig</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Quast.N50</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Quast.Total length</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Quast.Total length (&gt;= 0 bp)</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Quast.all_checks_passed</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Speciator.all_checks_passed</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Speciator.confidence</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Speciator.speciesName</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Sylph.all_checks_passed</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Sylph.number_of_genomes</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Sylph.top_species</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>Sylph.top_taxonomic_abundance</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>all_checks_passed</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>qualibact_compat_tier</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>qualibact_compat_passed</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>Checkm.Total_Contigs</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
         <is>
           <t>qualibact_compat_reasons</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>qualibact_compat_warn_policy</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>qualibact_compat_source</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>qualibact_compat_metrics_evaluated</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>qualibact_compat_metrics_missing</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>overall_qc</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>species</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>species_confidence</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>reason_summary</t>
         </is>
       </c>
     </row>
@@ -1072,169 +1189,190 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>19474</v>
+      </c>
+      <c r="J2" t="n">
         <v>522</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
+        <v>4153626</v>
+      </c>
+      <c r="L2" t="n">
+        <v>50.8872</v>
+      </c>
+      <c r="M2" t="n">
         <v>100</v>
       </c>
-      <c r="J2" t="n">
+      <c r="N2" t="n">
         <v>0.25</v>
       </c>
-      <c r="K2" t="n">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>75</v>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>75</v>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AB2" t="n">
+        <v>522</v>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AD2" t="n">
         <v>50.8872</v>
       </c>
-      <c r="L2" t="n">
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AF2" t="n">
+        <v>69909</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>19474</v>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AI2" t="n">
         <v>4153626</v>
       </c>
-      <c r="M2" t="n">
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AL2" t="n">
+        <v>100</v>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AN2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AP2" t="n">
         <v>19474</v>
       </c>
-      <c r="N2" t="n">
+      <c r="AQ2" t="n">
+        <v>50.8872</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>4153626</v>
+      </c>
+      <c r="AS2" t="n">
         <v>4264</v>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
+      <c r="AT2" t="n">
         <v>522</v>
       </c>
-      <c r="Q2" t="n">
-        <v>50.8872</v>
-      </c>
-      <c r="R2" t="n">
-        <v>69909</v>
-      </c>
-      <c r="S2" t="n">
-        <v>19474</v>
-      </c>
-      <c r="T2" t="n">
-        <v>4153626</v>
-      </c>
-      <c r="U2" t="n">
-        <v>4153626</v>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="AA2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="AC2" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>warn-as-warn</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
         <is>
           <t>Pinned QualiBact scheme for Escherichia coli</t>
         </is>
       </c>
-      <c r="AJ2" t="n">
+      <c r="AW2" t="n">
         <v>8</v>
       </c>
-      <c r="AK2" t="n">
+      <c r="AX2" t="n">
         <v>0</v>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
-        </is>
       </c>
     </row>
     <row r="3">
@@ -1245,169 +1383,190 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>126621</v>
+      </c>
+      <c r="J3" t="n">
         <v>679</v>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
+        <v>5738641</v>
+      </c>
+      <c r="L3" t="n">
+        <v>50.5585</v>
+      </c>
+      <c r="M3" t="n">
         <v>100</v>
       </c>
-      <c r="J3" t="n">
+      <c r="N3" t="n">
         <v>0.4</v>
       </c>
-      <c r="K3" t="n">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>75</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>75</v>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AB3" t="n">
+        <v>679</v>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AD3" t="n">
         <v>50.5585</v>
       </c>
-      <c r="L3" t="n">
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AF3" t="n">
+        <v>312707</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>126621</v>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AI3" t="n">
         <v>5738641</v>
       </c>
-      <c r="M3" t="n">
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AL3" t="n">
+        <v>100</v>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AN3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AP3" t="n">
         <v>126621</v>
       </c>
-      <c r="N3" t="n">
+      <c r="AQ3" t="n">
+        <v>50.5585</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>5738641</v>
+      </c>
+      <c r="AS3" t="n">
         <v>6105</v>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
+      <c r="AT3" t="n">
         <v>679</v>
       </c>
-      <c r="Q3" t="n">
-        <v>50.5585</v>
-      </c>
-      <c r="R3" t="n">
-        <v>312707</v>
-      </c>
-      <c r="S3" t="n">
-        <v>126621</v>
-      </c>
-      <c r="T3" t="n">
-        <v>5738641</v>
-      </c>
-      <c r="U3" t="n">
-        <v>5738641</v>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="AA3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="AC3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AF3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
+      <c r="AU3" t="inlineStr">
         <is>
           <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>warn-as-warn</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
+      <c r="AV3" t="inlineStr">
         <is>
           <t>Pinned QualiBact scheme for Escherichia coli</t>
         </is>
       </c>
-      <c r="AJ3" t="n">
+      <c r="AW3" t="n">
         <v>8</v>
       </c>
-      <c r="AK3" t="n">
+      <c r="AX3" t="n">
         <v>0</v>
-      </c>
-      <c r="AL3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="AO3" t="inlineStr">
-        <is>
-          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -1421,7 +1580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1432,32 +1591,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Speciator</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Sylph</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Quast</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Checkm</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Quast</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Speciator</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Sylph</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>all_checks_passed</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>QC_PASS</t>
+          <t>QC</t>
         </is>
       </c>
     </row>
@@ -1469,32 +1623,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1506,32 +1655,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1775,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>qualibact_compat_tier</t>
+          <t>qualibact_qc</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1673,7 +1817,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sylph.top_taxonomic_abundance</t>
+          <t>Sylph.top_abundance_percent</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -1683,17 +1827,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>75</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1935,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Quast.Total length</t>
+          <t>Quast.Total length (&gt;= 0 bp)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1957,7 +2101,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Checkm.GC</t>
+          <t>Checkm.GC_Content</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1982,7 +2126,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Checkm.Genome size (bp)</t>
+          <t>Checkm.Genome_Size</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">

</xml_diff>

<commit_message>
Standardize QC outputs and complete the v1.3.0 report (#17)
* Standardize QC reports and complete release evidence

* Silence false-positive QC label security findings

* Use valid fixture in CLI integration test
</commit_message>
<xml_diff>
--- a/examples/qualibact_ecoli/fail_only/report/report.xlsx
+++ b/examples/qualibact_ecoli/fail_only/report/report.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,67 +436,87 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>all_checks_passed</t>
+          <t>speccheck_qc</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>qualibact_compat_tier</t>
+          <t>qualibact_qc</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>historical_qualibact_qc</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>reason_summary</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>species</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>species_confidence</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>n50</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>contigs</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>genome_size</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>gc_percent</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>completeness</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>contamination</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>top_species</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>top_abundance</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>reason_summary</t>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>top_abundance_percent</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>threshold_source</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>report_schema_version</t>
         </is>
       </c>
     </row>
@@ -513,7 +533,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -521,45 +541,53 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>19474</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>522</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>4153626</v>
       </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
         <v>50.8872</v>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>100</v>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>0.25</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="N2" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
+      <c r="Q2" t="n">
+        <v>75</v>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -576,7 +604,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -584,45 +612,53 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>126621</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
         <v>679</v>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>5738641</v>
       </c>
-      <c r="J3" t="n">
+      <c r="L3" t="n">
         <v>50.5585</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>100</v>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>0.4</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="N3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
+      <c r="Q3" t="n">
+        <v>75</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -637,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -653,67 +689,87 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>all_checks_passed</t>
+          <t>speccheck_qc</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>qualibact_compat_tier</t>
+          <t>qualibact_qc</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>historical_qualibact_qc</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>reason_summary</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>species</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>species_confidence</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>n50</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>contigs</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>genome_size</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>gc_percent</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>completeness</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>contamination</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>top_species</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>top_abundance</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>reason_summary</t>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>top_abundance_percent</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>threshold_source</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>report_schema_version</t>
         </is>
       </c>
     </row>
@@ -730,7 +786,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -738,45 +794,53 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>19474</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>522</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>4153626</v>
       </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
         <v>50.8872</v>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>100</v>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>0.25</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="N2" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
+      <c r="Q2" t="n">
+        <v>75</v>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -793,7 +857,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -801,45 +865,53 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>126621</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
         <v>679</v>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>5738641</v>
       </c>
-      <c r="J3" t="n">
+      <c r="L3" t="n">
         <v>50.5585</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>100</v>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>0.4</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="N3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
+      <c r="Q3" t="n">
+        <v>75</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -854,7 +926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO3"/>
+  <dimension ref="A1:AX3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -865,202 +937,247 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Checkm.Completeness.check</t>
+          <t>overall_qc</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Checkm.Contamination.check</t>
+          <t>speccheck_qc</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Quast.# contigs (&gt;= 0 bp).check</t>
+          <t>qualibact_qc</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Quast.GC (%).check</t>
+          <t>historical_qualibact_qc</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Quast.N50.check</t>
+          <t>reason_summary</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Quast.Total length (&gt;= 0 bp).check</t>
+          <t>species</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Checkm.# contigs</t>
+          <t>species_confidence</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>n50</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>contigs</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>genome_size</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>gc_percent</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>completeness</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>contamination</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>top_species</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>top_abundance_percent</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>threshold_source</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>report_schema_version</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Speciator.qc_status</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Speciator.confidence</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Speciator.speciesName</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Sylph.qc_status</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Sylph.number_of_genomes</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Sylph.top_abundance_percent</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Sylph.top_species</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Quast.qc_status</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Quast.# contigs (&gt;= 0 bp)</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Quast.# contigs (&gt;= 0 bp).status</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>Quast.GC (%)</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>Quast.GC (%).status</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Quast.Largest contig</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Quast.N50</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>Quast.N50.status</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>Quast.Total length (&gt;= 0 bp)</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>Quast.Total length (&gt;= 0 bp).status</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>Checkm.qc_status</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
           <t>Checkm.Completeness</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>Checkm.Completeness.status</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Checkm.Contamination</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Checkm.GC</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Checkm.Genome size (bp)</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Checkm.N50 (scaffolds)</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>Checkm.Contamination.status</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>Checkm.Contig_N50</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>Checkm.GC_Content</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>Checkm.Genome_Size</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
         <is>
           <t>Checkm.Total_Coding_Sequences</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Checkm.all_checks_passed</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Quast.# contigs (&gt;= 0 bp)</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Quast.GC (%)</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Quast.Largest contig</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Quast.N50</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Quast.Total length</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Quast.Total length (&gt;= 0 bp)</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Quast.all_checks_passed</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Speciator.all_checks_passed</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Speciator.confidence</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Speciator.speciesName</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Sylph.all_checks_passed</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Sylph.number_of_genomes</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Sylph.top_species</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>Sylph.top_taxonomic_abundance</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>all_checks_passed</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>qualibact_compat_tier</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>qualibact_compat_passed</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>Checkm.Total_Contigs</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
         <is>
           <t>qualibact_compat_reasons</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>qualibact_compat_warn_policy</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>qualibact_compat_source</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>qualibact_compat_metrics_evaluated</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>qualibact_compat_metrics_missing</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>overall_qc</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>species</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>species_confidence</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>reason_summary</t>
         </is>
       </c>
     </row>
@@ -1072,169 +1189,190 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>19474</v>
+      </c>
+      <c r="J2" t="n">
         <v>522</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
+        <v>4153626</v>
+      </c>
+      <c r="L2" t="n">
+        <v>50.8872</v>
+      </c>
+      <c r="M2" t="n">
         <v>100</v>
       </c>
-      <c r="J2" t="n">
+      <c r="N2" t="n">
         <v>0.25</v>
       </c>
-      <c r="K2" t="n">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>75</v>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>75</v>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AB2" t="n">
+        <v>522</v>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AD2" t="n">
         <v>50.8872</v>
       </c>
-      <c r="L2" t="n">
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AF2" t="n">
+        <v>69909</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>19474</v>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AI2" t="n">
         <v>4153626</v>
       </c>
-      <c r="M2" t="n">
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AL2" t="n">
+        <v>100</v>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AN2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AP2" t="n">
         <v>19474</v>
       </c>
-      <c r="N2" t="n">
+      <c r="AQ2" t="n">
+        <v>50.8872</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>4153626</v>
+      </c>
+      <c r="AS2" t="n">
         <v>4264</v>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
+      <c r="AT2" t="n">
         <v>522</v>
       </c>
-      <c r="Q2" t="n">
-        <v>50.8872</v>
-      </c>
-      <c r="R2" t="n">
-        <v>69909</v>
-      </c>
-      <c r="S2" t="n">
-        <v>19474</v>
-      </c>
-      <c r="T2" t="n">
-        <v>4153626</v>
-      </c>
-      <c r="U2" t="n">
-        <v>4153626</v>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="AA2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="AC2" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>warn-as-warn</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
         <is>
           <t>Pinned QualiBact scheme for Escherichia coli</t>
         </is>
       </c>
-      <c r="AJ2" t="n">
+      <c r="AW2" t="n">
         <v>8</v>
       </c>
-      <c r="AK2" t="n">
+      <c r="AX2" t="n">
         <v>0</v>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
-        </is>
       </c>
     </row>
     <row r="3">
@@ -1245,169 +1383,190 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>126621</v>
+      </c>
+      <c r="J3" t="n">
         <v>679</v>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
+        <v>5738641</v>
+      </c>
+      <c r="L3" t="n">
+        <v>50.5585</v>
+      </c>
+      <c r="M3" t="n">
         <v>100</v>
       </c>
-      <c r="J3" t="n">
+      <c r="N3" t="n">
         <v>0.4</v>
       </c>
-      <c r="K3" t="n">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>75</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="X3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>75</v>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AB3" t="n">
+        <v>679</v>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AD3" t="n">
         <v>50.5585</v>
       </c>
-      <c r="L3" t="n">
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AF3" t="n">
+        <v>312707</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>126621</v>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AI3" t="n">
         <v>5738641</v>
       </c>
-      <c r="M3" t="n">
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AL3" t="n">
+        <v>100</v>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AN3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="AP3" t="n">
         <v>126621</v>
       </c>
-      <c r="N3" t="n">
+      <c r="AQ3" t="n">
+        <v>50.5585</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>5738641</v>
+      </c>
+      <c r="AS3" t="n">
         <v>6105</v>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
+      <c r="AT3" t="n">
         <v>679</v>
       </c>
-      <c r="Q3" t="n">
-        <v>50.5585</v>
-      </c>
-      <c r="R3" t="n">
-        <v>312707</v>
-      </c>
-      <c r="S3" t="n">
-        <v>126621</v>
-      </c>
-      <c r="T3" t="n">
-        <v>5738641</v>
-      </c>
-      <c r="U3" t="n">
-        <v>5738641</v>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="AA3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="AC3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AF3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
+      <c r="AU3" t="inlineStr">
         <is>
           <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>warn-as-warn</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
+      <c r="AV3" t="inlineStr">
         <is>
           <t>Pinned QualiBact scheme for Escherichia coli</t>
         </is>
       </c>
-      <c r="AJ3" t="n">
+      <c r="AW3" t="n">
         <v>8</v>
       </c>
-      <c r="AK3" t="n">
+      <c r="AX3" t="n">
         <v>0</v>
-      </c>
-      <c r="AL3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="AO3" t="inlineStr">
-        <is>
-          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -1421,7 +1580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1432,32 +1591,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Speciator</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Sylph</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Quast</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Checkm</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Quast</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Speciator</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Sylph</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>all_checks_passed</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>QC_PASS</t>
+          <t>QC</t>
         </is>
       </c>
     </row>
@@ -1469,32 +1623,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1506,32 +1655,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1775,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>qualibact_compat_tier</t>
+          <t>qualibact_qc</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1673,7 +1817,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sylph.top_taxonomic_abundance</t>
+          <t>Sylph.top_abundance_percent</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -1683,17 +1827,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>75</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1935,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Quast.Total length</t>
+          <t>Quast.Total length (&gt;= 0 bp)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1957,7 +2101,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Checkm.GC</t>
+          <t>Checkm.GC_Content</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1982,7 +2126,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Checkm.Genome size (bp)</t>
+          <t>Checkm.Genome_Size</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">

</xml_diff>